<commit_message>
Deployed 94200fa with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/downloads/acces-structure-editoriale.xlsx
+++ b/downloads/acces-structure-editoriale.xlsx
@@ -453,14 +453,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Éditeur privé</t>
+          <t>Organisme public de recherche</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="C2" t="n">
-        <v>67</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -479,40 +479,40 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Organisme public de recherche</t>
+          <t>Association</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Association</t>
+          <t>Coédition éditeur privé &amp; structure publique ou associative</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Coédition éditeur privé &amp; structure publique ou associative</t>
+          <t>Éditeur privé</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>